<commit_message>
Updated startup sets size 4
</commit_message>
<xml_diff>
--- a/src/data/clean_data_new.xlsx
+++ b/src/data/clean_data_new.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\OneDrive\Documents\GitHub\ExperimentEH\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{4E61CB91-9F18-4BFA-A133-1A110597D4E1}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A8E44E1-3393-4528-926B-E29B25464045}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="13_ncr:1_{4E61CB91-9F18-4BFA-A133-1A110597D4E1}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8B09C1C-577C-44F2-8EF7-CA687EADD9B1}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="startup" sheetId="1" r:id="rId1"/>
@@ -326,8 +326,7 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-We randomize a 6-name set out of 8 choices and so have variations in composition, i.e. 1, 2, or 3 females in the set.
-For randomization, create a separate dataset with the 8 values.</t>
+In pilot2 we have a set of 4 startups with one female and 3 male. The order is randomized.</t>
         </r>
       </text>
     </comment>
@@ -361,8 +360,7 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-We randomize this information across the 7 options. Then will also have variations in composition, e.g. 3-3 external-internal or 4-2 external-internal.
-For randomization, create a separate dataset with the 7 values.</t>
+In pilot 2, for 4-startup set, we keep the list of 3 external evaluators and 2 self evaluation. Thus also have variations in set composition: 3-1 or 2-2 ext-self.</t>
         </r>
       </text>
     </comment>
@@ -371,7 +369,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="51">
   <si>
     <t>Startup_name_altered</t>
   </si>
@@ -443,9 +441,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Venture capital firm New Enterprise Associates estimated the start-up’s value at </t>
-  </si>
-  <si>
     <t>The start-up valuation is based on the founder’s long-term growth outlook, estimating it at</t>
   </si>
   <si>
@@ -470,18 +465,6 @@
     <t>Noah</t>
   </si>
   <si>
-    <t>Paul</t>
-  </si>
-  <si>
-    <t>Sarah</t>
-  </si>
-  <si>
-    <t>Nancy</t>
-  </si>
-  <si>
-    <t>Jack</t>
-  </si>
-  <si>
     <t>Valuation_amount</t>
   </si>
   <si>
@@ -534,9 +517,6 @@
   </si>
   <si>
     <t>Venture capital firm Sequoia set a pre-money valuation of the start-up at</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Using internal performance indicators, the founder estimates the start-up's value at  </t>
   </si>
   <si>
     <t>The start-up specializes in regenerative medicine, developing a novel biological platform that replaces and regenerates body tissues.</t>
@@ -952,7 +932,7 @@
   <sheetFormatPr defaultColWidth="48.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" customWidth="1"/>
     <col min="3" max="3" width="48.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="41.5703125" style="4" customWidth="1"/>
     <col min="5" max="5" width="13.7109375" style="4" customWidth="1"/>
@@ -975,13 +955,13 @@
         <v>2</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>4</v>
@@ -999,22 +979,22 @@
         <v>7</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="E2" s="4">
         <v>2018</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="G2" s="4">
         <v>35</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="I2" s="4"/>
     </row>
@@ -1026,22 +1006,22 @@
         <v>9</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="E3" s="4">
         <v>2020</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G3" s="4">
         <v>34</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="I3" s="4"/>
     </row>
@@ -1053,22 +1033,22 @@
         <v>11</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E4" s="4">
         <v>2016</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="G4" s="4">
         <v>35</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="I4" s="4"/>
     </row>
@@ -1080,22 +1060,22 @@
         <v>13</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="E5" s="4">
         <v>2018</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="G5" s="4">
         <v>35</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="I5" s="4"/>
     </row>
@@ -1107,22 +1087,22 @@
         <v>15</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="E6" s="4">
         <v>2017</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="G6" s="4">
         <v>27</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="I6" s="4"/>
     </row>
@@ -1134,22 +1114,22 @@
         <v>17</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="E7" s="4">
         <v>2023</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="G7" s="4">
         <v>27</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="I7" s="4"/>
     </row>
@@ -1223,7 +1203,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{059E7891-9034-456E-AB36-CA10D5237DC2}">
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.5703125" style="4" customWidth="1"/>
@@ -1231,48 +1211,40 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>30</v>
-      </c>
+      <c r="A8" s="6"/>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>31</v>
-      </c>
+      <c r="A9" s="6"/>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="6"/>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6"/>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="6"/>
@@ -1282,18 +1254,6 @@
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="6"/>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="6"/>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="6"/>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="6"/>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1303,7 +1263,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B129C1FF-A6A4-4674-8988-1354FBDEAAA7}">
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="41.5703125" style="4" customWidth="1"/>
@@ -1319,12 +1279,12 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>20</v>
       </c>
@@ -1336,18 +1296,14 @@
     </row>
     <row r="6" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>50</v>
-      </c>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="6"/>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6"/>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="6"/>
@@ -1363,12 +1319,6 @@
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="6"/>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="6"/>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated startup json and investment page for set4
</commit_message>
<xml_diff>
--- a/src/data/clean_data_new.xlsx
+++ b/src/data/clean_data_new.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\OneDrive\Documents\GitHub\ExperimentEH\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="13_ncr:1_{4E61CB91-9F18-4BFA-A133-1A110597D4E1}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8B09C1C-577C-44F2-8EF7-CA687EADD9B1}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{4E61CB91-9F18-4BFA-A133-1A110597D4E1}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E98584B-FC54-4AB5-8EE8-5865BC3D001F}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -326,7 +326,8 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-In pilot2 we have a set of 4 startups with one female and 3 male. The order is randomized.</t>
+We randomize a 6-name set out of 8 choices and so have variations in composition, i.e. 1, 2, or 3 females in the set.
+For randomization, create a separate dataset with the 8 values.</t>
         </r>
       </text>
     </comment>
@@ -360,7 +361,8 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-In pilot 2, for 4-startup set, we keep the list of 3 external evaluators and 2 self evaluation. Thus also have variations in set composition: 3-1 or 2-2 ext-self.</t>
+We randomize this information across the 7 options. Then will also have variations in composition, e.g. 3-3 external-internal or 4-2 external-internal.
+For randomization, create a separate dataset with the 7 values.</t>
         </r>
       </text>
     </comment>
@@ -369,7 +371,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="58">
   <si>
     <t>Startup_name_altered</t>
   </si>
@@ -441,7 +443,7 @@
     </r>
   </si>
   <si>
-    <t>The start-up valuation is based on the founder’s long-term growth outlook, estimating it at</t>
+    <t xml:space="preserve">Venture capital firm New Enterprise Associates estimated the start-up’s value at </t>
   </si>
   <si>
     <t xml:space="preserve">JPMorgan Chase Innovation Banking valued the start-up at </t>
@@ -465,6 +467,18 @@
     <t>Noah</t>
   </si>
   <si>
+    <t>Paul</t>
+  </si>
+  <si>
+    <t>Sarah</t>
+  </si>
+  <si>
+    <t>Nancy</t>
+  </si>
+  <si>
+    <t>Jack</t>
+  </si>
+  <si>
     <t>Valuation_amount</t>
   </si>
   <si>
@@ -516,7 +530,7 @@
     <t>Thompson</t>
   </si>
   <si>
-    <t>Venture capital firm Sequoia set a pre-money valuation of the start-up at</t>
+    <t xml:space="preserve">Using internal performance indicators, the founder estimates the start-up's value at  </t>
   </si>
   <si>
     <t>The start-up specializes in regenerative medicine, developing a novel biological platform that replaces and regenerates body tissues.</t>
@@ -535,6 +549,15 @@
   </si>
   <si>
     <t>The start-up offers a new credit card solution designed to move small dollar loan customers into a more affordable product.</t>
+  </si>
+  <si>
+    <t>gender</t>
+  </si>
+  <si>
+    <t>female</t>
+  </si>
+  <si>
+    <t>male</t>
   </si>
 </sst>
 </file>
@@ -932,7 +955,7 @@
   <sheetFormatPr defaultColWidth="48.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.28515625" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="48.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="41.5703125" style="4" customWidth="1"/>
     <col min="5" max="5" width="13.7109375" style="4" customWidth="1"/>
@@ -955,13 +978,13 @@
         <v>2</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>4</v>
@@ -979,22 +1002,22 @@
         <v>7</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E2" s="4">
         <v>2018</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="G2" s="4">
         <v>35</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="I2" s="4"/>
     </row>
@@ -1006,22 +1029,22 @@
         <v>9</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E3" s="4">
         <v>2020</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="G3" s="4">
         <v>34</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="I3" s="4"/>
     </row>
@@ -1033,22 +1056,22 @@
         <v>11</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="E4" s="4">
         <v>2016</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="G4" s="4">
         <v>35</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="I4" s="4"/>
     </row>
@@ -1060,22 +1083,22 @@
         <v>13</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E5" s="4">
         <v>2018</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G5" s="4">
         <v>35</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="I5" s="4"/>
     </row>
@@ -1087,22 +1110,22 @@
         <v>15</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="E6" s="4">
         <v>2017</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="G6" s="4">
         <v>27</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="I6" s="4"/>
     </row>
@@ -1114,22 +1137,22 @@
         <v>17</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="E7" s="4">
         <v>2023</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="G7" s="4">
         <v>27</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="I7" s="4"/>
     </row>
@@ -1203,57 +1226,104 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{059E7891-9034-456E-AB36-CA10D5237DC2}">
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.5703125" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="6"/>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6"/>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="6"/>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6"/>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="6"/>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="6"/>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="6"/>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="6"/>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="6"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="6"/>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1279,7 +1349,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>19</v>
       </c>
@@ -1296,7 +1366,7 @@
     </row>
     <row r="6" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated startup sets and nudge info
</commit_message>
<xml_diff>
--- a/src/data/clean_data_new.xlsx
+++ b/src/data/clean_data_new.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\OneDrive\Documents\GitHub\ExperimentEH\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{4E61CB91-9F18-4BFA-A133-1A110597D4E1}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E98584B-FC54-4AB5-8EE8-5865BC3D001F}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{4E61CB91-9F18-4BFA-A133-1A110597D4E1}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{2733D4D8-6A4A-4A3D-8D43-680C5C0B0DA6}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="startup" sheetId="1" r:id="rId1"/>
@@ -371,7 +371,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="59">
   <si>
     <t>Startup_name_altered</t>
   </si>
@@ -558,6 +558,9 @@
   </si>
   <si>
     <t>male</t>
+  </si>
+  <si>
+    <t>The start-up valuation is based on the founder’s long-term growth outlook, estimating it at</t>
   </si>
 </sst>
 </file>
@@ -1369,6 +1372,11 @@
         <v>48</v>
       </c>
     </row>
+    <row r="7" spans="1:1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="6"/>
     </row>

</xml_diff>

<commit_message>
Startup set 6 without evaluation, news 2 options
</commit_message>
<xml_diff>
--- a/src/data/clean_data_new.xlsx
+++ b/src/data/clean_data_new.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\OneDrive\Documents\GitHub\ExperimentEH\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{4E61CB91-9F18-4BFA-A133-1A110597D4E1}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A8E44E1-3393-4528-926B-E29B25464045}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="113_{B6C4C99A-F10F-4828-9BFB-B8097B1364CE}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{400182F3-E6C9-4AE5-AFDF-01155384EB94}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="startup" sheetId="1" r:id="rId1"/>
@@ -326,8 +326,8 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-We randomize a 6-name set out of 8 choices and so have variations in composition, i.e. 1, 2, or 3 females in the set.
-For randomization, create a separate dataset with the 8 values.</t>
+We randomize a 6-name set out of 7 choices and so have variations in composition, i.e. 1 or 2 females in the set.
+For randomization, create a separate dataset with the 7 values.</t>
         </r>
       </text>
     </comment>
@@ -371,7 +371,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="56">
   <si>
     <t>Startup_name_altered</t>
   </si>
@@ -458,30 +458,12 @@
     <t>Founder_firstname_altered</t>
   </si>
   <si>
-    <t xml:space="preserve">Jessica </t>
-  </si>
-  <si>
     <t>William</t>
   </si>
   <si>
-    <t>George</t>
-  </si>
-  <si>
-    <t>Noah</t>
-  </si>
-  <si>
-    <t>Paul</t>
-  </si>
-  <si>
     <t>Sarah</t>
   </si>
   <si>
-    <t>Nancy</t>
-  </si>
-  <si>
-    <t>Jack</t>
-  </si>
-  <si>
     <t>Valuation_amount</t>
   </si>
   <si>
@@ -527,9 +509,6 @@
     <t>Founded_10</t>
   </si>
   <si>
-    <t>Miles</t>
-  </si>
-  <si>
     <t>Thompson</t>
   </si>
   <si>
@@ -555,6 +534,24 @@
   </si>
   <si>
     <t>The start-up offers a new credit card solution designed to move small dollar loan customers into a more affordable product.</t>
+  </si>
+  <si>
+    <t>Jessica</t>
+  </si>
+  <si>
+    <t>Michael</t>
+  </si>
+  <si>
+    <t>Jacob</t>
+  </si>
+  <si>
+    <t>Daniel</t>
+  </si>
+  <si>
+    <t>Steven</t>
+  </si>
+  <si>
+    <t>Briggs</t>
   </si>
 </sst>
 </file>
@@ -975,13 +972,13 @@
         <v>2</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>4</v>
@@ -999,22 +996,22 @@
         <v>7</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="E2" s="4">
         <v>2018</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="G2" s="4">
         <v>35</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="I2" s="4"/>
     </row>
@@ -1026,22 +1023,22 @@
         <v>9</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="E3" s="4">
         <v>2020</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="G3" s="4">
         <v>34</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="I3" s="4"/>
     </row>
@@ -1053,22 +1050,22 @@
         <v>11</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E4" s="4">
         <v>2016</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="G4" s="4">
         <v>35</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="I4" s="4"/>
     </row>
@@ -1080,22 +1077,22 @@
         <v>13</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="E5" s="4">
         <v>2018</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="G5" s="4">
         <v>35</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="I5" s="4"/>
     </row>
@@ -1107,22 +1104,22 @@
         <v>15</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="E6" s="4">
         <v>2017</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="G6" s="4">
         <v>27</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="I6" s="4"/>
     </row>
@@ -1134,22 +1131,22 @@
         <v>17</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="E7" s="4">
         <v>2023</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="G7" s="4">
         <v>27</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="I7" s="4"/>
     </row>
@@ -1235,43 +1232,38 @@
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>31</v>
+      <c r="A8" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
@@ -1341,12 +1333,12 @@
     </row>
     <row r="7" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated startup card content
</commit_message>
<xml_diff>
--- a/src/data/clean_data_new.xlsx
+++ b/src/data/clean_data_new.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\OneDrive\Documents\GitHub\ExperimentEH\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="113_{B6C4C99A-F10F-4828-9BFB-B8097B1364CE}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{400182F3-E6C9-4AE5-AFDF-01155384EB94}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="109_{39B5942E-0A98-4489-83CA-FE968D0092B1}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{81FE0972-1497-4E31-8089-5C0A132B82F2}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="startup" sheetId="1" r:id="rId1"/>
@@ -371,7 +371,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="54">
   <si>
     <t>Startup_name_altered</t>
   </si>
@@ -512,9 +512,6 @@
     <t>Thompson</t>
   </si>
   <si>
-    <t>Venture capital firm Sequoia set a pre-money valuation of the start-up at</t>
-  </si>
-  <si>
     <t xml:space="preserve">Using internal performance indicators, the founder estimates the start-up's value at  </t>
   </si>
   <si>
@@ -546,9 +543,6 @@
   </si>
   <si>
     <t>Daniel</t>
-  </si>
-  <si>
-    <t>Steven</t>
   </si>
   <si>
     <t>Briggs</t>
@@ -996,7 +990,7 @@
         <v>7</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>27</v>
@@ -1023,7 +1017,7 @@
         <v>9</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>28</v>
@@ -1050,7 +1044,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>29</v>
@@ -1077,7 +1071,7 @@
         <v>13</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>30</v>
@@ -1104,7 +1098,7 @@
         <v>15</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>31</v>
@@ -1131,7 +1125,7 @@
         <v>17</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>32</v>
@@ -1140,7 +1134,7 @@
         <v>2023</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G7" s="4">
         <v>27</v>
@@ -1233,7 +1227,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -1243,17 +1237,17 @@
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
@@ -1262,9 +1256,7 @@
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>54</v>
-      </c>
+      <c r="A8"/>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="6"/>
@@ -1295,7 +1287,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B129C1FF-A6A4-4674-8988-1354FBDEAAA7}">
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="41.5703125" style="4" customWidth="1"/>
@@ -1336,10 +1328,8 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>43</v>
-      </c>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6"/>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="6"/>
@@ -1358,9 +1348,6 @@
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="6"/>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Replaced valuation with performance indicator in startup sets
</commit_message>
<xml_diff>
--- a/src/data/clean_data_new.xlsx
+++ b/src/data/clean_data_new.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\OneDrive\Documents\GitHub\ExperimentEH\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="109_{39B5942E-0A98-4489-83CA-FE968D0092B1}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{81FE0972-1497-4E31-8089-5C0A132B82F2}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="109_{39B5942E-0A98-4489-83CA-FE968D0092B1}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF553786-91EB-41D4-91F1-36AC03BC96B5}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="startup" sheetId="1" r:id="rId1"/>
     <sheet name="founder" sheetId="2" r:id="rId2"/>
     <sheet name="value" sheetId="3" r:id="rId3"/>
+    <sheet name="indicator" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="179021"/>
   <extLst>
@@ -370,8 +371,42 @@
 </comments>
 </file>
 
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>admin</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{19357E93-694D-459A-A9FF-572094B2AD08}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>admin:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+3 unverifiable and 3 verifiable</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="61">
   <si>
     <t>Startup_name_altered</t>
   </si>
@@ -546,6 +581,27 @@
   </si>
   <si>
     <t>Briggs</t>
+  </si>
+  <si>
+    <t>performance_indicator</t>
+  </si>
+  <si>
+    <t>The founder reports positive internal employee satisfaction and a highly motivated team.</t>
+  </si>
+  <si>
+    <t>The founder highlights strong revenue momentum over the past year, pointing to encouraging growth.</t>
+  </si>
+  <si>
+    <t>The start-up completed a successful third-party product trial with positive feedback from customers and industry analysts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The start-up’s recent funding rounds include strategic investments from JPMorgan Chase and Sequoia Capital. </t>
+  </si>
+  <si>
+    <t>In recognition of its technology innovation, the start-up was selected for the Google for Startups Accelerator.</t>
+  </si>
+  <si>
+    <t>According to the founder, the start-up is seeing greater market reach and increased visibility in key tech media.</t>
   </si>
 </sst>
 </file>
@@ -1353,4 +1409,53 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17E5BA47-CBF1-4F08-9E4D-A758848525C3}">
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="126.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Cleaned startup json n=120 and news json n=120
</commit_message>
<xml_diff>
--- a/src/data/clean_data_new.xlsx
+++ b/src/data/clean_data_new.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\OneDrive\Documents\GitHub\ExperimentEH\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="109_{39B5942E-0A98-4489-83CA-FE968D0092B1}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF553786-91EB-41D4-91F1-36AC03BC96B5}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="109_{39B5942E-0A98-4489-83CA-FE968D0092B1}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{62537CAC-6B69-4DDD-AF23-3D5823FC9BD0}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="startup" sheetId="1" r:id="rId1"/>
@@ -589,19 +589,19 @@
     <t>The founder reports positive internal employee satisfaction and a highly motivated team.</t>
   </si>
   <si>
-    <t>The founder highlights strong revenue momentum over the past year, pointing to encouraging growth.</t>
-  </si>
-  <si>
     <t>The start-up completed a successful third-party product trial with positive feedback from customers and industry analysts.</t>
   </si>
   <si>
-    <t xml:space="preserve">The start-up’s recent funding rounds include strategic investments from JPMorgan Chase and Sequoia Capital. </t>
-  </si>
-  <si>
-    <t>In recognition of its technology innovation, the start-up was selected for the Google for Startups Accelerator.</t>
-  </si>
-  <si>
-    <t>According to the founder, the start-up is seeing greater market reach and increased visibility in key tech media.</t>
+    <t>According to its website, the start-up is seeing great market reach and increased visibility in the media.</t>
+  </si>
+  <si>
+    <t>The start-up's updates highlight strong revenue momentum over the past year, pointing to encouraging growth.</t>
+  </si>
+  <si>
+    <t>After a competitive review, the start-up’s technology was validated through selection into the Google for Startups Accelerator.</t>
+  </si>
+  <si>
+    <t>The start-up secured investments from JPMorgan Chase and Sequoia Capital following rigorous expert due diligence.</t>
   </si>
 </sst>
 </file>
@@ -996,22 +996,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L18"/>
-  <sheetFormatPr defaultColWidth="48.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="48.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="48.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="41.5703125" style="4" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" style="4" customWidth="1"/>
-    <col min="6" max="6" width="14.85546875" style="4" customWidth="1"/>
-    <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.140625" style="4" customWidth="1"/>
-    <col min="9" max="9" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="41.5546875" style="4" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="14.88671875" style="4" customWidth="1"/>
+    <col min="7" max="7" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.109375" style="4" customWidth="1"/>
+    <col min="9" max="9" width="20.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="17.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="I1" s="1"/>
     </row>
-    <row r="2" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>6</v>
       </c>
@@ -1065,7 +1065,7 @@
       </c>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>8</v>
       </c>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="I3" s="4"/>
     </row>
-    <row r="4" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>10</v>
       </c>
@@ -1119,7 +1119,7 @@
       </c>
       <c r="I4" s="4"/>
     </row>
-    <row r="5" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>12</v>
       </c>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="I5" s="4"/>
     </row>
-    <row r="6" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>14</v>
       </c>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="I6" s="4"/>
     </row>
-    <row r="7" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>16</v>
       </c>
@@ -1200,7 +1200,7 @@
       </c>
       <c r="I7" s="4"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -1210,7 +1210,7 @@
       <c r="K8" s="4"/>
       <c r="L8" s="4"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -1220,43 +1220,43 @@
       <c r="K9" s="4"/>
       <c r="L9" s="4"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
       <c r="F12" s="6"/>
       <c r="H12" s="6"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
       <c r="F13" s="6"/>
       <c r="H13" s="6"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
       <c r="F14" s="6"/>
       <c r="H14" s="6"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D15" s="6"/>
       <c r="E15" s="6"/>
       <c r="F15" s="6"/>
       <c r="H15" s="6"/>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D16" s="6"/>
       <c r="E16" s="6"/>
       <c r="F16" s="6"/>
       <c r="H16" s="6"/>
     </row>
-    <row r="17" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
       <c r="H17" s="6"/>
     </row>
-    <row r="18" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="4:8" x14ac:dyDescent="0.3">
       <c r="D18" s="6"/>
       <c r="E18" s="6"/>
       <c r="F18" s="6"/>
@@ -1271,68 +1271,68 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{059E7891-9034-456E-AB36-CA10D5237DC2}">
   <dimension ref="A1:A18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.5703125" style="4" customWidth="1"/>
+    <col min="1" max="1" width="27.5546875" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8"/>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="6"/>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" s="6"/>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" s="6"/>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" s="6"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" s="6"/>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" s="6"/>
     </row>
   </sheetData>
@@ -1344,65 +1344,65 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B129C1FF-A6A4-4674-8988-1354FBDEAAA7}">
   <dimension ref="A1:A17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="41.5703125" style="4" customWidth="1"/>
+    <col min="1" max="1" width="41.5546875" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="6"/>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="6"/>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="6"/>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" s="6"/>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" s="6"/>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" s="6"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" s="6"/>
     </row>
   </sheetData>
@@ -1414,44 +1414,44 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17E5BA47-CBF1-4F08-9E4D-A758848525C3}">
   <dimension ref="A1:A7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="126.28515625" customWidth="1"/>
+    <col min="1" max="1" width="111.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Removed experience and evaluation info from startup sets and updated instruction
</commit_message>
<xml_diff>
--- a/src/data/clean_data_new.xlsx
+++ b/src/data/clean_data_new.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\OneDrive\Documents\GitHub\ExperimentEH\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="113_{B6C4C99A-F10F-4828-9BFB-B8097B1364CE}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{400182F3-E6C9-4AE5-AFDF-01155384EB94}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="6_{00044203-FB9A-42BA-A111-77D48916F293}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CDB083D-4755-4032-A604-8E87B3137828}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="startup" sheetId="1" r:id="rId1"/>
     <sheet name="founder" sheetId="2" r:id="rId2"/>
     <sheet name="value" sheetId="3" r:id="rId3"/>
+    <sheet name="indicator" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="179021"/>
   <extLst>
@@ -370,8 +371,42 @@
 </comments>
 </file>
 
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>admin</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{ED2320DF-EB8D-454C-B1F7-6AA858409493}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>admin:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+3 unverifiable and 3 verifiable</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="64">
   <si>
     <t>Startup_name_altered</t>
   </si>
@@ -458,9 +493,6 @@
     <t>Founder_firstname_altered</t>
   </si>
   <si>
-    <t>William</t>
-  </si>
-  <si>
     <t>Sarah</t>
   </si>
   <si>
@@ -494,9 +526,6 @@
     <t>Shelton</t>
   </si>
   <si>
-    <t>Krueger</t>
-  </si>
-  <si>
     <t>Hayden</t>
   </si>
   <si>
@@ -536,22 +565,52 @@
     <t>The start-up offers a new credit card solution designed to move small dollar loan customers into a more affordable product.</t>
   </si>
   <si>
-    <t>Jessica</t>
-  </si>
-  <si>
-    <t>Michael</t>
-  </si>
-  <si>
-    <t>Jacob</t>
-  </si>
-  <si>
     <t>Daniel</t>
   </si>
   <si>
-    <t>Steven</t>
-  </si>
-  <si>
-    <t>Briggs</t>
+    <t>Miles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jessica </t>
+  </si>
+  <si>
+    <t>Brandon</t>
+  </si>
+  <si>
+    <t>Ryan</t>
+  </si>
+  <si>
+    <t>Amanda</t>
+  </si>
+  <si>
+    <t>Jack</t>
+  </si>
+  <si>
+    <t>Eric</t>
+  </si>
+  <si>
+    <t>performance_indicator</t>
+  </si>
+  <si>
+    <t>The founder reports positive internal employee satisfaction and a highly motivated team.</t>
+  </si>
+  <si>
+    <t>The start-up's updates highlight strong revenue momentum over the past year, pointing to encouraging growth.</t>
+  </si>
+  <si>
+    <t>According to its website, the start-up is seeing great market reach and increased visibility in the media.</t>
+  </si>
+  <si>
+    <t>The start-up completed a successful third-party product trial with positive feedback from customers and industry analysts.</t>
+  </si>
+  <si>
+    <t>After a competitive review, the start-up’s technology was validated through selection into the Google for Startups Accelerator.</t>
+  </si>
+  <si>
+    <t>The start-up secured investments from JPMorgan Chase and Sequoia Capital following rigorous expert due diligence.</t>
+  </si>
+  <si>
+    <t>Parker</t>
   </si>
 </sst>
 </file>
@@ -972,13 +1031,13 @@
         <v>2</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>4</v>
@@ -996,22 +1055,22 @@
         <v>7</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E2" s="4">
         <v>2018</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G2" s="4">
         <v>35</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="I2" s="4"/>
     </row>
@@ -1023,22 +1082,22 @@
         <v>9</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E3" s="4">
         <v>2020</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G3" s="4">
         <v>34</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="I3" s="4"/>
     </row>
@@ -1050,22 +1109,22 @@
         <v>11</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E4" s="4">
         <v>2016</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G4" s="4">
         <v>35</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="I4" s="4"/>
     </row>
@@ -1077,22 +1136,22 @@
         <v>13</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E5" s="4">
         <v>2018</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>36</v>
+        <v>63</v>
       </c>
       <c r="G5" s="4">
         <v>35</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="I5" s="4"/>
     </row>
@@ -1104,22 +1163,22 @@
         <v>15</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E6" s="4">
         <v>2017</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G6" s="4">
         <v>27</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="I6" s="4"/>
     </row>
@@ -1131,22 +1190,22 @@
         <v>17</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E7" s="4">
         <v>2023</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="G7" s="4">
         <v>27</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="I7" s="4"/>
     </row>
@@ -1232,37 +1291,42 @@
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="4" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>25</v>
+      <c r="A3" s="4" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4" s="4" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="A5" s="4" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="A6" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1333,12 +1397,12 @@
     </row>
     <row r="7" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
@@ -1361,6 +1425,55 @@
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="6"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF065494-C4AB-4E77-8FEC-CA80D10A1E37}">
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="116" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>62</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added valuation info back in
</commit_message>
<xml_diff>
--- a/src/data/clean_data_new.xlsx
+++ b/src/data/clean_data_new.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\OneDrive\Documents\GitHub\ExperimentEH\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="6_{00044203-FB9A-42BA-A111-77D48916F293}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CDB083D-4755-4032-A604-8E87B3137828}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="6_{00044203-FB9A-42BA-A111-77D48916F293}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{3F1861AE-06E2-418C-9B56-48ED1B0D89D8}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="startup" sheetId="1" r:id="rId1"/>
@@ -233,7 +233,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>admin:</t>
         </r>
@@ -242,7 +242,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 increase from 2016</t>
@@ -257,7 +257,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>admin:</t>
         </r>
@@ -266,7 +266,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 increase from original 2011 to match lowest founder age</t>
@@ -281,7 +281,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>admin:</t>
         </r>
@@ -290,7 +290,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 increase from 2015</t>
@@ -385,7 +385,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>admin:</t>
         </r>
@@ -394,7 +394,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 3 unverifiable and 3 verifiable</t>
@@ -406,7 +406,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="65">
   <si>
     <t>Startup_name_altered</t>
   </si>
@@ -478,18 +478,9 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Venture capital firm New Enterprise Associates estimated the start-up’s value at </t>
-  </si>
-  <si>
-    <t>The start-up valuation is based on the founder’s long-term growth outlook, estimating it at</t>
-  </si>
-  <si>
     <t xml:space="preserve">JPMorgan Chase Innovation Banking valued the start-up at </t>
   </si>
   <si>
-    <t>According to the founder’s internal valuation model, the business is worth</t>
-  </si>
-  <si>
     <t>Founder_firstname_altered</t>
   </si>
   <si>
@@ -541,9 +532,6 @@
     <t>Thompson</t>
   </si>
   <si>
-    <t>Venture capital firm Sequoia set a pre-money valuation of the start-up at</t>
-  </si>
-  <si>
     <t xml:space="preserve">Using internal performance indicators, the founder estimates the start-up's value at  </t>
   </si>
   <si>
@@ -592,32 +580,187 @@
     <t>performance_indicator</t>
   </si>
   <si>
-    <t>The founder reports positive internal employee satisfaction and a highly motivated team.</t>
-  </si>
-  <si>
-    <t>The start-up's updates highlight strong revenue momentum over the past year, pointing to encouraging growth.</t>
-  </si>
-  <si>
-    <t>According to its website, the start-up is seeing great market reach and increased visibility in the media.</t>
-  </si>
-  <si>
-    <t>The start-up completed a successful third-party product trial with positive feedback from customers and industry analysts.</t>
-  </si>
-  <si>
-    <t>After a competitive review, the start-up’s technology was validated through selection into the Google for Startups Accelerator.</t>
-  </si>
-  <si>
-    <t>The start-up secured investments from JPMorgan Chase and Sequoia Capital following rigorous expert due diligence.</t>
-  </si>
-  <si>
     <t>Parker</t>
+  </si>
+  <si>
+    <t>The start-up valuation is based on the founder’s growth outlook, estimating it at</t>
+  </si>
+  <si>
+    <t>According to the founder’s valuation model, the business is worth</t>
+  </si>
+  <si>
+    <t>Venture capital firm Sequoia set an estimated valuation of the start-up at</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Venture capital firm New Enterprise Associates estimated the start-up’s worth at </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Website information:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The start-up reports strong employee satisfaction and a highly motivated team.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Website information:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The start-up highlights 2x revenue growth over the past year.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Website information:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The start-up reports increased market reach and growing visibility in the media.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Third-party validation:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The start-up received positive feedback from customers and analysts in a recent product trial.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Third-party validation:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The start-up was selected for the Google for Startups Accelerator after an in-depth review.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Third-party validation:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The start-up completed due diligence and secured investment from JPMorgan Chase.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Third-party validation:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The start-up was technically vetted by industry experts and funded by Sequoia Capital.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -653,19 +796,6 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1031,13 +1161,13 @@
         <v>2</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>4</v>
@@ -1055,22 +1185,22 @@
         <v>7</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E2" s="4">
         <v>2018</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="G2" s="4">
         <v>35</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="I2" s="4"/>
     </row>
@@ -1082,22 +1212,22 @@
         <v>9</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E3" s="4">
         <v>2020</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G3" s="4">
         <v>34</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="I3" s="4"/>
     </row>
@@ -1109,22 +1239,22 @@
         <v>11</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E4" s="4">
         <v>2016</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="G4" s="4">
         <v>35</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="I4" s="4"/>
     </row>
@@ -1136,22 +1266,22 @@
         <v>13</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E5" s="4">
         <v>2018</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="G5" s="4">
         <v>35</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="I5" s="4"/>
     </row>
@@ -1163,22 +1293,22 @@
         <v>15</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E6" s="4">
         <v>2017</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="G6" s="4">
         <v>27</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="I6" s="4"/>
     </row>
@@ -1190,22 +1320,22 @@
         <v>17</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E7" s="4">
         <v>2023</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G7" s="4">
         <v>27</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="I7" s="4"/>
     </row>
@@ -1287,47 +1417,47 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
@@ -1362,7 +1492,7 @@
   <dimension ref="A1:A18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="41.5703125" style="4" customWidth="1"/>
+    <col min="1" max="1" width="85.7109375" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1370,39 +1500,39 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
@@ -1434,45 +1564,50 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF065494-C4AB-4E77-8FEC-CA80D10A1E37}">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="116" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="105" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>62</v>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Replaced valuation with performance indicator and reformatted
</commit_message>
<xml_diff>
--- a/src/data/clean_data_new.xlsx
+++ b/src/data/clean_data_new.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\OneDrive\Documents\GitHub\ExperimentEH\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="6_{00044203-FB9A-42BA-A111-77D48916F293}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{3F1861AE-06E2-418C-9B56-48ED1B0D89D8}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="6_{00044203-FB9A-42BA-A111-77D48916F293}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{50B61064-0946-4F0E-A559-D25303B56BB6}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -604,7 +604,30 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Website information:</t>
+      <t>Highlight from third-party source:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The start-up received positive feedback from customers and analysts in a recent product trial.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Highlight from start-up website:</t>
     </r>
     <r>
       <rPr>
@@ -627,76 +650,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Website information:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The start-up highlights 2x revenue growth over the past year.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Website information:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The start-up reports increased market reach and growing visibility in the media.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Third-party validation:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The start-up received positive feedback from customers and analysts in a recent product trial.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Third-party validation:</t>
+      <t>Highlight from third-party source:</t>
     </r>
     <r>
       <rPr>
@@ -719,7 +673,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Third-party validation:</t>
+      <t>Highlight from third-party source:</t>
     </r>
     <r>
       <rPr>
@@ -742,7 +696,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Third-party validation:</t>
+      <t>Highlight from third-party source:</t>
     </r>
     <r>
       <rPr>
@@ -753,6 +707,52 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> The start-up was technically vetted by industry experts and funded by Sequoia Capital.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Highlight from start-up website:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The start-up reports a twofold increase in its revenue over the past year.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Highlight from start-up website:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The start-up reports a broader market reach and greater visibility in the media.</t>
     </r>
   </si>
 </sst>
@@ -1567,7 +1567,7 @@
   <dimension ref="A1:A8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="105" customWidth="1"/>
+    <col min="1" max="1" width="116.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="45" x14ac:dyDescent="0.25">
@@ -1577,37 +1577,37 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added info to raw startup data
</commit_message>
<xml_diff>
--- a/src/data/clean_data_new.xlsx
+++ b/src/data/clean_data_new.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\OneDrive\Documents\GitHub\ExperimentEH\src\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cec8835d7d99e403/Documents/GitHub/ExperimentEH/src/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="6_{00044203-FB9A-42BA-A111-77D48916F293}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{50B61064-0946-4F0E-A559-D25303B56BB6}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="6_{00044203-FB9A-42BA-A111-77D48916F293}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{A649D4A7-AE26-46DF-9B63-74435747A12A}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="startup" sheetId="1" r:id="rId1"/>
@@ -406,7 +406,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="68">
   <si>
     <t>Startup_name_altered</t>
   </si>
@@ -754,6 +754,15 @@
       </rPr>
       <t xml:space="preserve"> The start-up reports a broader market reach and greater visibility in the media.</t>
     </r>
+  </si>
+  <si>
+    <t>Founder_prefix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ms. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mr. </t>
   </si>
 </sst>
 </file>
@@ -1409,70 +1418,98 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{059E7891-9034-456E-AB36-CA10D5237DC2}">
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.5703125" style="4" customWidth="1"/>
+    <col min="2" max="2" width="27.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="6"/>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="6"/>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="6"/>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="6"/>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="6"/>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Added review info with ms mr
</commit_message>
<xml_diff>
--- a/src/data/clean_data_new.xlsx
+++ b/src/data/clean_data_new.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\OneDrive\Documents\GitHub\ExperimentEH\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="6_{00044203-FB9A-42BA-A111-77D48916F293}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{3F1861AE-06E2-418C-9B56-48ED1B0D89D8}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="113_{233005F1-386F-4933-844A-E6CECC66C7D2}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C8AE059-BB9A-44D4-879C-C97CDA82AC99}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="startup" sheetId="1" r:id="rId1"/>
     <sheet name="founder" sheetId="2" r:id="rId2"/>
-    <sheet name="value" sheetId="3" r:id="rId3"/>
-    <sheet name="indicator" sheetId="4" r:id="rId4"/>
+    <sheet name="review" sheetId="5" r:id="rId3"/>
+    <sheet name="value" sheetId="3" r:id="rId4"/>
+    <sheet name="indicator" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="179021"/>
   <extLst>
@@ -406,7 +407,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="75">
   <si>
     <t>Startup_name_altered</t>
   </si>
@@ -754,6 +755,36 @@
       </rPr>
       <t xml:space="preserve"> The start-up was technically vetted by industry experts and funded by Sequoia Capital.</t>
     </r>
+  </si>
+  <si>
+    <t>Founder_prefix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ms. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mr. </t>
+  </si>
+  <si>
+    <t>Review_status</t>
+  </si>
+  <si>
+    <t>According to the founder, the product meets enterprise-grade standards.</t>
+  </si>
+  <si>
+    <t>The product has passed technology tests conducted by the founder's expert team.</t>
+  </si>
+  <si>
+    <t>Based on the founder's report, the product is qualified for market launch.</t>
+  </si>
+  <si>
+    <t>The product has been technically validated by external industry specialists.</t>
+  </si>
+  <si>
+    <t>The product has been reviewed and validated by Goldman Sachs' tech division.</t>
+  </si>
+  <si>
+    <t>The product has undergone due diligence and been approved by third-party auditors.</t>
   </si>
 </sst>
 </file>
@@ -1409,70 +1440,97 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{059E7891-9034-456E-AB36-CA10D5237DC2}">
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.5703125" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="6"/>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="6"/>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="6"/>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="6"/>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="6"/>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
@@ -1488,6 +1546,54 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEF97743-4886-4B04-BB26-93A63D18FCE6}">
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="181.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B129C1FF-A6A4-4674-8988-1354FBDEAAA7}">
   <dimension ref="A1:A18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1562,7 +1668,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF065494-C4AB-4E77-8FEC-CA80D10A1E37}">
   <dimension ref="A1:A8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Replaced valuation with founder pitch
</commit_message>
<xml_diff>
--- a/src/data/clean_data_new.xlsx
+++ b/src/data/clean_data_new.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\OneDrive\Documents\GitHub\ExperimentEH\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{4E61CB91-9F18-4BFA-A133-1A110597D4E1}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A8E44E1-3393-4528-926B-E29B25464045}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{4E61CB91-9F18-4BFA-A133-1A110597D4E1}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{F859B754-8773-4D61-B42B-5FD1567B49A3}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="startup" sheetId="1" r:id="rId1"/>
     <sheet name="founder" sheetId="2" r:id="rId2"/>
     <sheet name="value" sheetId="3" r:id="rId3"/>
+    <sheet name="pitch" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="179021"/>
   <extLst>
@@ -232,7 +233,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>admin:</t>
         </r>
@@ -241,7 +242,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 increase from 2016</t>
@@ -256,7 +257,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>admin:</t>
         </r>
@@ -265,7 +266,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 increase from original 2011 to match lowest founder age</t>
@@ -280,7 +281,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>admin:</t>
         </r>
@@ -289,7 +290,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 increase from 2015</t>
@@ -371,7 +372,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="70">
   <si>
     <t>Startup_name_altered</t>
   </si>
@@ -556,12 +557,51 @@
   <si>
     <t>The start-up offers a new credit card solution designed to move small dollar loan customers into a more affordable product.</t>
   </si>
+  <si>
+    <t>Founder_pitch</t>
+  </si>
+  <si>
+    <t>Our innovation promises the next leap for future biotechnology.</t>
+  </si>
+  <si>
+    <t>Our technology is certified by external experts after more than 20 clinical trials.</t>
+  </si>
+  <si>
+    <t>We redefine the skies for enterprise by leading industrial intelligence.</t>
+  </si>
+  <si>
+    <t>Our drones passed over 30 quality tests with positive feedback from clients and analysts.</t>
+  </si>
+  <si>
+    <t>Set to become a market leader, we transform every product into a connection.</t>
+  </si>
+  <si>
+    <t>After 15+ pilots, our platform has shown reliable product-to-app integration.</t>
+  </si>
+  <si>
+    <t>In the vast digital world, we are the first to tell brands where it's best to be seen.</t>
+  </si>
+  <si>
+    <t>Our product has been offered to 50+ clients and records stable revenue growth.</t>
+  </si>
+  <si>
+    <t>We disrupt telehealth with a solution for scale, speed, and smart care delivery.</t>
+  </si>
+  <si>
+    <t>Following extensive third-party testing, our product is ready to benefit people's health.</t>
+  </si>
+  <si>
+    <t>We’re not just launching a card; we’re launching a movement.</t>
+  </si>
+  <si>
+    <t>External specialists have validated the technical feasibility of our credit model.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -598,19 +638,6 @@
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -644,7 +671,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -668,6 +695,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1374,4 +1402,122 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EB6DF7F-14B9-4AFE-8AEE-A4A43919E4D7}">
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="23.42578125" customWidth="1"/>
+    <col min="2" max="2" width="82.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Generated sets with 3 pairs of diff genders
</commit_message>
<xml_diff>
--- a/src/data/clean_data_new.xlsx
+++ b/src/data/clean_data_new.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\OneDrive\Documents\GitHub\ExperimentEH\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{4E61CB91-9F18-4BFA-A133-1A110597D4E1}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A8E44E1-3393-4528-926B-E29B25464045}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="109_{03CF3122-DFFA-4B79-8846-078C30F8C8F5}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="startup" sheetId="1" r:id="rId1"/>
@@ -232,7 +232,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>admin:</t>
         </r>
@@ -241,7 +241,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 increase from 2016</t>
@@ -256,7 +256,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>admin:</t>
         </r>
@@ -265,7 +265,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 increase from original 2011 to match lowest founder age</t>
@@ -280,7 +280,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>admin:</t>
         </r>
@@ -289,7 +289,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 increase from 2015</t>
@@ -371,7 +371,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="62">
   <si>
     <t>Startup_name_altered</t>
   </si>
@@ -556,12 +556,27 @@
   <si>
     <t>The start-up offers a new credit card solution designed to move small dollar loan customers into a more affordable product.</t>
   </si>
+  <si>
+    <t>gender</t>
+  </si>
+  <si>
+    <t>female</t>
+  </si>
+  <si>
+    <t>male</t>
+  </si>
+  <si>
+    <t>Amanda</t>
+  </si>
+  <si>
+    <t>Megan</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -597,19 +612,6 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1223,70 +1225,113 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{059E7891-9034-456E-AB36-CA10D5237DC2}">
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.5703125" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="6"/>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="6"/>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="6"/>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="6"/>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="6"/>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated content for pair setup
</commit_message>
<xml_diff>
--- a/src/data/clean_data_new.xlsx
+++ b/src/data/clean_data_new.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\OneDrive\Documents\GitHub\ExperimentEH\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="109_{03CF3122-DFFA-4B79-8846-078C30F8C8F5}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="109_{03CF3122-DFFA-4B79-8846-078C30F8C8F5}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{2ACB34C3-5BA9-415F-86F7-C103B7E9BD3F}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="startup" sheetId="1" r:id="rId1"/>
@@ -371,7 +371,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="60">
   <si>
     <t>Startup_name_altered</t>
   </si>
@@ -564,12 +564,6 @@
   </si>
   <si>
     <t>male</t>
-  </si>
-  <si>
-    <t>Amanda</t>
-  </si>
-  <si>
-    <t>Megan</t>
   </si>
 </sst>
 </file>
@@ -1225,7 +1219,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{059E7891-9034-456E-AB36-CA10D5237DC2}">
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.5703125" style="4" customWidth="1"/>
@@ -1304,20 +1298,10 @@
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="B10" t="s">
-        <v>58</v>
-      </c>
+      <c r="A10" s="6"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="B11" t="s">
-        <v>58</v>
-      </c>
+      <c r="A11" s="6"/>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="6"/>
@@ -1333,12 +1317,6 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="6"/>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="6"/>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>